<commit_message>
Pierwsze przymiarki do plytki
</commit_message>
<xml_diff>
--- a/ESP_MCP_I2C/pomiary_I2C.xlsx
+++ b/ESP_MCP_I2C/pomiary_I2C.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafal\Desktop\studia II st\praca magisterska\ESP_MCP_I2C\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A531B016-513D-42BC-9378-0158E9294483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A9AFE68-2C90-443A-8181-7E2F453C74D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15225" yWindow="1515" windowWidth="21600" windowHeight="11295" xr2:uid="{1AA4BAB9-C97F-426F-B328-BA28CD04F64C}"/>
+    <workbookView xWindow="6810" yWindow="2925" windowWidth="21600" windowHeight="11295" xr2:uid="{1AA4BAB9-C97F-426F-B328-BA28CD04F64C}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="14">
   <si>
     <t>długość kabla [m]</t>
   </si>
@@ -69,7 +69,13 @@
     <t>dla I2C</t>
   </si>
   <si>
-    <t>nie działa</t>
+    <t>dla I2C pomaranczowy- SDA</t>
+  </si>
+  <si>
+    <t>Niebieski - SCL</t>
+  </si>
+  <si>
+    <t>zaczyna się psuć (czasami po resecie działa)</t>
   </si>
 </sst>
 </file>
@@ -94,7 +100,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -102,13 +108,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -423,127 +446,838 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6496F60A-78B9-4FFB-A9C0-B981B64B8CC7}">
-  <dimension ref="B1:E12"/>
+  <dimension ref="B1:H89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.85546875" customWidth="1"/>
     <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="8" max="8" width="21.140625" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1">
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="C4" s="3">
         <v>100000</v>
       </c>
-      <c r="D4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="D4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="C5" s="3">
         <v>1000000</v>
       </c>
-      <c r="D5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1">
+      <c r="D5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="C6" s="3">
         <v>1100000</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="C7" s="3">
         <v>1250000</v>
       </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" s="1">
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="C8" s="3">
         <v>1500000</v>
       </c>
-      <c r="D8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1">
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="C9" s="3">
         <v>2500000</v>
       </c>
-      <c r="D9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10" s="1">
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="C10" s="3">
         <v>5000000</v>
       </c>
-      <c r="D10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12">
-        <v>5.5</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>11</v>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C15" s="3">
+        <v>100000</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C16" s="3">
+        <v>200000</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="3">
+        <v>300000</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C18" s="3">
+        <v>400000</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C19" s="3">
+        <v>500000</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C20" s="3">
+        <v>600000</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C21" s="3">
+        <v>700000</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C22" s="3">
+        <v>800000</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C23" s="3">
+        <v>900000</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C24" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="H25" s="1"/>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="2">
+        <v>1</v>
+      </c>
+      <c r="C31" s="3">
+        <v>100000</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" s="2">
+        <v>1</v>
+      </c>
+      <c r="C32" s="3">
+        <v>200000</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B33" s="2">
+        <v>1</v>
+      </c>
+      <c r="C33" s="3">
+        <v>300000</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B34" s="2">
+        <v>1</v>
+      </c>
+      <c r="C34" s="3">
+        <v>400000</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B35" s="2">
+        <v>1</v>
+      </c>
+      <c r="C35" s="3">
+        <v>500000</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="2">
+        <v>1</v>
+      </c>
+      <c r="C36" s="3">
+        <v>600000</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+      <c r="C37" s="3">
+        <v>700000</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B38" s="2">
+        <v>1</v>
+      </c>
+      <c r="C38" s="3">
+        <v>800000</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B39" s="2">
+        <v>1</v>
+      </c>
+      <c r="C39" s="3">
+        <v>900000</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B40" s="2">
+        <v>1</v>
+      </c>
+      <c r="C40" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B45" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B46" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B47" s="2">
+        <v>2</v>
+      </c>
+      <c r="C47" s="3">
+        <v>100000</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B48" s="2">
+        <v>2</v>
+      </c>
+      <c r="C48" s="3">
+        <v>200000</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B49" s="2">
+        <v>2</v>
+      </c>
+      <c r="C49" s="3">
+        <v>300000</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B50" s="2">
+        <v>2</v>
+      </c>
+      <c r="C50" s="3">
+        <v>400000</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B51" s="2">
+        <v>2</v>
+      </c>
+      <c r="C51" s="3">
+        <v>500000</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B52" s="2">
+        <v>2</v>
+      </c>
+      <c r="C52" s="3">
+        <v>600000</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B53" s="2">
+        <v>2</v>
+      </c>
+      <c r="C53" s="3">
+        <v>700000</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B54" s="2">
+        <v>2</v>
+      </c>
+      <c r="C54" s="3">
+        <v>800000</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B55" s="2">
+        <v>2</v>
+      </c>
+      <c r="C55" s="3">
+        <v>900000</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B56" s="2">
+        <v>2</v>
+      </c>
+      <c r="C56" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B57" s="2">
+        <v>2</v>
+      </c>
+      <c r="C57" s="3">
+        <v>1100000</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B58" s="2">
+        <v>2</v>
+      </c>
+      <c r="C58" s="3">
+        <v>1200000</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B61" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B62" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B63" s="2">
+        <v>3</v>
+      </c>
+      <c r="C63" s="3">
+        <v>100000</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B64" s="2">
+        <v>3</v>
+      </c>
+      <c r="C64" s="3">
+        <v>200000</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B65" s="2">
+        <v>3</v>
+      </c>
+      <c r="C65" s="3">
+        <v>300000</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B66" s="2">
+        <v>3</v>
+      </c>
+      <c r="C66" s="3">
+        <v>400000</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B67" s="2">
+        <v>3</v>
+      </c>
+      <c r="C67" s="3">
+        <v>500000</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B68" s="2">
+        <v>3</v>
+      </c>
+      <c r="C68" s="3">
+        <v>600000</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B69" s="2">
+        <v>3</v>
+      </c>
+      <c r="C69" s="3">
+        <v>700000</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B70" s="2">
+        <v>3</v>
+      </c>
+      <c r="C70" s="3">
+        <v>800000</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B71" s="2">
+        <v>3</v>
+      </c>
+      <c r="C71" s="3">
+        <v>900000</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B72" s="2">
+        <v>3</v>
+      </c>
+      <c r="C72" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B73" s="2">
+        <v>3</v>
+      </c>
+      <c r="C73" s="3">
+        <v>1100000</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B77" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="78" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B78" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B79" s="2">
+        <v>5</v>
+      </c>
+      <c r="C79" s="3">
+        <v>100000</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B80" s="2">
+        <v>5</v>
+      </c>
+      <c r="C80" s="3">
+        <v>200000</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B81" s="2">
+        <v>5</v>
+      </c>
+      <c r="C81" s="3">
+        <v>300000</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B82" s="2">
+        <v>5</v>
+      </c>
+      <c r="C82" s="3">
+        <v>400000</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B83" s="2">
+        <v>5</v>
+      </c>
+      <c r="C83" s="3">
+        <v>500000</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="84" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B84" s="2">
+        <v>5</v>
+      </c>
+      <c r="C84" s="3">
+        <v>600000</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="85" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B85" s="2">
+        <v>5</v>
+      </c>
+      <c r="C85" s="3">
+        <v>700000</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B86" s="2">
+        <v>5</v>
+      </c>
+      <c r="C86" s="3">
+        <v>800000</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="87" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B87" s="2">
+        <v>5</v>
+      </c>
+      <c r="C87" s="3">
+        <v>900000</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B88" s="2">
+        <v>5</v>
+      </c>
+      <c r="C88" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="89" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B89" s="2">
+        <v>5</v>
+      </c>
+      <c r="C89" s="3">
+        <v>1100000</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>